<commit_message>
update: submit status for profs
</commit_message>
<xml_diff>
--- a/sample-data/professors.xlsx
+++ b/sample-data/professors.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Professors" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:B2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -406,68 +406,18 @@
       <c r="B1" t="str">
         <v>email</v>
       </c>
-      <c r="C1" t="str">
-        <v>password</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Dr. Rajesh Kumar</v>
+        <v>Dr. Test Professor</v>
       </c>
       <c r="B2" t="str">
-        <v>rajesh.kumar@iiti.ac.in</v>
-      </c>
-      <c r="C2" t="str">
-        <v>prof123</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Dr. Priya Sharma</v>
-      </c>
-      <c r="B3" t="str">
-        <v>priya.sharma@iiti.ac.in</v>
-      </c>
-      <c r="C3" t="str">
-        <v>prof123</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Dr. Amit Verma</v>
-      </c>
-      <c r="B4" t="str">
-        <v>amit.verma@iiti.ac.in</v>
-      </c>
-      <c r="C4" t="str">
-        <v>prof123</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Dr. Sunita Patel</v>
-      </c>
-      <c r="B5" t="str">
-        <v>sunita.patel@iiti.ac.in</v>
-      </c>
-      <c r="C5" t="str">
-        <v>prof123</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Dr. Vikram Singh</v>
-      </c>
-      <c r="B6" t="str">
-        <v>vikram.singh@iiti.ac.in</v>
-      </c>
-      <c r="C6" t="str">
-        <v>prof123</v>
+        <v>test.prof@iiti.ac.in</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>